<commit_message>
Update generated reference workbooks (customer inventory, test data)
Binary workbook changes already in the working tree; not regenerated or reviewed in this change.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/VFQ_DXP_Test_Data_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/VFQ_DXP_Test_Data_Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_9F580439F813B7AA711314D825925AC49123B7BE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D529B64C-F105-EC4D-9CFF-11126A8CDEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1340" windowWidth="34560" windowHeight="21000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="20400" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -40,12 +40,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ID Lookup (MOI Fetch)'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Persona by Approach'!$A$1:$F$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="806">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="810">
   <si>
     <t>Staff ID</t>
   </si>
@@ -1172,72 +1172,48 @@
     <t>Customer</t>
   </si>
   <si>
-    <t>Ahmed, Fatima, CUST-1003</t>
-  </si>
-  <si>
     <t>Name or customer ID (QID, mobile and email are searched on the Customer Search page).</t>
   </si>
   <si>
     <t>Lead</t>
   </si>
   <si>
-    <t>LEAD-20001, MNP, Home</t>
-  </si>
-  <si>
     <t>Lead ID or service needed.</t>
   </si>
   <si>
     <t>Trouble ticket</t>
   </si>
   <si>
-    <t>TT-40001, Mobile Complaints</t>
-  </si>
-  <si>
     <t>Ticket ID or category.</t>
   </si>
   <si>
     <t>Order</t>
   </si>
   <si>
-    <t>ORD-90001, Postpaid, FWA</t>
-  </si>
-  <si>
     <t>Order ID or order type.</t>
   </si>
   <si>
     <t>SIM swap</t>
   </si>
   <si>
-    <t>SSW-6601, +97433001001</t>
-  </si>
-  <si>
     <t>SIM swap order ID or mobile number.</t>
   </si>
   <si>
     <t>Catalogue item</t>
   </si>
   <si>
-    <t>CAT-1001, or a product name</t>
-  </si>
-  <si>
     <t>Name or catalogue ID.</t>
   </si>
   <si>
     <t>Campaign</t>
   </si>
   <si>
-    <t>CMP-MNP-0819, Cross-sell, Postpaid upgrade</t>
-  </si>
-  <si>
     <t>Campaign name or ID.</t>
   </si>
   <si>
     <t>Screen or module</t>
   </si>
   <si>
-    <t>Checkout, SCR-037</t>
-  </si>
-  <si>
     <t>Screen names and screen IDs also show up as navigation results.</t>
   </si>
   <si>
@@ -2463,15 +2439,58 @@
   </si>
   <si>
     <t>Applies to both Forgot Password reset and in-session Change Password.</t>
+  </si>
+  <si>
+    <t>Ahmed</t>
+  </si>
+  <si>
+    <t>Fatima</t>
+  </si>
+  <si>
+    <t>Postpaid</t>
+  </si>
+  <si>
+    <t>FWA</t>
+  </si>
+  <si>
+    <t>SSW-6601</t>
+  </si>
+  <si>
+    <t>CAT-1001</t>
+  </si>
+  <si>
+    <t>product name</t>
+  </si>
+  <si>
+    <t>CMP-MNP-0819</t>
+  </si>
+  <si>
+    <t>Cross-sell</t>
+  </si>
+  <si>
+    <t>Postpaid upgrade</t>
+  </si>
+  <si>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>SCR-037</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2554,6 +2573,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -2610,7 +2643,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -2661,12 +2694,64 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </left>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </left>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </left>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </left>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2674,7 +2759,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2683,37 +2768,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2731,101 +2816,128 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3141,20 +3253,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26" customHeight="1">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="61" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
     </row>
     <row r="4" spans="1:4" ht="28" customHeight="1">
       <c r="A4" s="16" t="s">
@@ -3360,76 +3472,76 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>371</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>491</v>
+        <v>483</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>334</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>347</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>334</v>
@@ -3440,16 +3552,16 @@
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>334</v>
@@ -3460,16 +3572,16 @@
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>347</v>
@@ -3480,36 +3592,36 @@
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>334</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>511</v>
+        <v>503</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>512</v>
+        <v>504</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>347</v>
@@ -3520,16 +3632,16 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>513</v>
+        <v>505</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>514</v>
+        <v>506</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>515</v>
+        <v>507</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>334</v>
@@ -3540,36 +3652,36 @@
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>517</v>
+        <v>509</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>334</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>334</v>
@@ -3606,54 +3718,54 @@
   <sheetData>
     <row r="1" spans="1:9" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>318</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>349</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>191</v>
@@ -3664,28 +3776,28 @@
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>354</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>515</v>
+        <v>507</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="I3" s="4">
         <v>24</v>
@@ -3693,28 +3805,28 @@
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>341</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>529</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>541</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>542</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>537</v>
-      </c>
       <c r="H4" s="4" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="I4" s="4">
         <v>48</v>
@@ -3722,28 +3834,28 @@
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>357</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>515</v>
+        <v>507</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="I5" s="4">
         <v>24</v>
@@ -3751,28 +3863,28 @@
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>361</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="I6" s="4">
         <v>24</v>
@@ -3780,55 +3892,55 @@
     </row>
     <row r="9" spans="1:9" ht="17" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>550</v>
+        <v>542</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>551</v>
+        <v>543</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>553</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="30" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="30" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
     </row>
   </sheetData>
@@ -3855,87 +3967,87 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>318</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>349</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>564</v>
+        <v>556</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>354</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>566</v>
+        <v>558</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>567</v>
+        <v>559</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>349</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>569</v>
+        <v>561</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>191</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>570</v>
+        <v>562</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>571</v>
+        <v>563</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>341</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>572</v>
+        <v>564</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -3961,44 +4073,44 @@
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>574</v>
+        <v>566</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>577</v>
+        <v>569</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>580</v>
+        <v>572</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>581</v>
+        <v>573</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
     </row>
   </sheetData>
@@ -4025,59 +4137,59 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>585</v>
+        <v>577</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>587</v>
+        <v>579</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>322</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>588</v>
+        <v>580</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>589</v>
+        <v>581</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>591</v>
+        <v>583</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>592</v>
+        <v>584</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>191</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>593</v>
+        <v>585</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>596</v>
+        <v>588</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>597</v>
+        <v>589</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>598</v>
+        <v>590</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>191</v>
@@ -4107,44 +4219,44 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18">
       <c r="A1" s="50" t="s">
-        <v>599</v>
+        <v>591</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16">
       <c r="A2" s="51" t="s">
-        <v>600</v>
+        <v>592</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>601</v>
+        <v>593</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="112">
       <c r="A3" s="49" t="s">
-        <v>602</v>
+        <v>594</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>603</v>
+        <v>595</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="176">
       <c r="A4" s="49" t="s">
-        <v>604</v>
+        <v>596</v>
       </c>
       <c r="B4" s="49" t="s">
-        <v>605</v>
+        <v>597</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="160">
       <c r="A5" s="49" t="s">
-        <v>606</v>
+        <v>598</v>
       </c>
       <c r="B5" s="49" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="36">
       <c r="A7" s="50" t="s">
-        <v>608</v>
+        <v>600</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16">
@@ -4158,136 +4270,136 @@
         <v>322</v>
       </c>
       <c r="D8" s="51" t="s">
-        <v>585</v>
+        <v>577</v>
       </c>
       <c r="E8" s="51" t="s">
-        <v>609</v>
+        <v>601</v>
       </c>
       <c r="F8" s="51" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="G8" s="51" t="s">
-        <v>610</v>
+        <v>602</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="32">
       <c r="A9" s="49" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="B9" s="49" t="s">
         <v>349</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>612</v>
+        <v>604</v>
       </c>
       <c r="D9" s="49" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="E9" s="49" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="F9" s="49" t="s">
-        <v>591</v>
+        <v>583</v>
       </c>
       <c r="G9" s="49" t="s">
-        <v>614</v>
+        <v>606</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16">
       <c r="A10" s="49" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="B10" s="49" t="s">
         <v>354</v>
       </c>
       <c r="C10" s="49" t="s">
-        <v>616</v>
+        <v>608</v>
       </c>
       <c r="D10" s="49" t="s">
-        <v>617</v>
+        <v>609</v>
       </c>
       <c r="E10" s="49" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="F10" s="49" t="s">
-        <v>596</v>
+        <v>588</v>
       </c>
       <c r="G10" s="49" t="s">
-        <v>618</v>
+        <v>610</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16">
       <c r="A11" s="49" t="s">
-        <v>619</v>
+        <v>611</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>620</v>
+        <v>612</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="D11" s="49" t="s">
-        <v>622</v>
+        <v>614</v>
       </c>
       <c r="E11" s="49" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="F11" s="49" t="s">
-        <v>623</v>
+        <v>615</v>
       </c>
       <c r="G11" s="49" t="s">
-        <v>624</v>
+        <v>616</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16">
       <c r="A12" s="49" t="s">
-        <v>625</v>
+        <v>617</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>626</v>
+        <v>618</v>
       </c>
       <c r="C12" s="49" t="s">
-        <v>627</v>
+        <v>619</v>
       </c>
       <c r="D12" s="49" t="s">
-        <v>628</v>
+        <v>620</v>
       </c>
       <c r="E12" s="49" t="s">
         <v>322</v>
       </c>
       <c r="F12" s="49" t="s">
-        <v>591</v>
+        <v>583</v>
       </c>
       <c r="G12" s="49" t="s">
-        <v>629</v>
+        <v>621</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16">
       <c r="A13" s="49" t="s">
-        <v>630</v>
+        <v>622</v>
       </c>
       <c r="B13" s="49" t="s">
         <v>357</v>
       </c>
       <c r="C13" s="49" t="s">
-        <v>631</v>
+        <v>623</v>
       </c>
       <c r="D13" s="49" t="s">
-        <v>632</v>
+        <v>624</v>
       </c>
       <c r="E13" s="49" t="s">
-        <v>633</v>
+        <v>625</v>
       </c>
       <c r="F13" s="49" t="s">
-        <v>634</v>
+        <v>626</v>
       </c>
       <c r="G13" s="49" t="s">
-        <v>635</v>
+        <v>627</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="36">
       <c r="A15" s="50" t="s">
-        <v>636</v>
+        <v>628</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16">
@@ -4298,10 +4410,10 @@
         <v>318</v>
       </c>
       <c r="C16" s="51" t="s">
-        <v>637</v>
+        <v>629</v>
       </c>
       <c r="D16" s="51" t="s">
-        <v>638</v>
+        <v>630</v>
       </c>
       <c r="E16" s="51" t="s">
         <v>322</v>
@@ -4312,67 +4424,67 @@
     </row>
     <row r="17" spans="1:8" ht="32">
       <c r="A17" s="49" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="B17" s="49" t="s">
         <v>349</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>639</v>
+        <v>631</v>
       </c>
       <c r="D17" s="49" t="s">
-        <v>640</v>
+        <v>632</v>
       </c>
       <c r="E17" s="49" t="s">
-        <v>641</v>
+        <v>633</v>
       </c>
       <c r="F17" s="49" t="s">
-        <v>642</v>
+        <v>634</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="32">
       <c r="A18" s="49" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="B18" s="49" t="s">
         <v>354</v>
       </c>
       <c r="C18" s="49" t="s">
-        <v>643</v>
+        <v>635</v>
       </c>
       <c r="D18" s="49" t="s">
-        <v>644</v>
+        <v>636</v>
       </c>
       <c r="E18" s="49" t="s">
-        <v>645</v>
+        <v>637</v>
       </c>
       <c r="F18" s="49" t="s">
-        <v>646</v>
+        <v>638</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="32">
       <c r="A19" s="49" t="s">
-        <v>619</v>
+        <v>611</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>620</v>
+        <v>612</v>
       </c>
       <c r="C19" s="49" t="s">
-        <v>647</v>
+        <v>639</v>
       </c>
       <c r="D19" s="49" t="s">
-        <v>648</v>
+        <v>640</v>
       </c>
       <c r="E19" s="49" t="s">
-        <v>649</v>
+        <v>641</v>
       </c>
       <c r="F19" s="49" t="s">
-        <v>650</v>
+        <v>642</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="36">
       <c r="A21" s="50" t="s">
-        <v>651</v>
+        <v>643</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="16">
@@ -4383,183 +4495,183 @@
         <v>318</v>
       </c>
       <c r="C22" s="51" t="s">
-        <v>652</v>
+        <v>644</v>
       </c>
       <c r="D22" s="51" t="s">
-        <v>653</v>
+        <v>645</v>
       </c>
       <c r="E22" s="51" t="s">
-        <v>654</v>
+        <v>646</v>
       </c>
       <c r="F22" s="51" t="s">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="G22" s="51" t="s">
-        <v>656</v>
+        <v>648</v>
       </c>
       <c r="H22" s="51" t="s">
-        <v>657</v>
+        <v>649</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="32">
       <c r="A23" s="49" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="B23" s="49" t="s">
         <v>349</v>
       </c>
       <c r="C23" s="49" t="s">
-        <v>658</v>
+        <v>650</v>
       </c>
       <c r="D23" s="49" t="s">
-        <v>659</v>
+        <v>651</v>
       </c>
       <c r="E23" s="49" t="s">
         <v>347</v>
       </c>
       <c r="F23" s="49" t="s">
-        <v>660</v>
+        <v>652</v>
       </c>
       <c r="G23" s="49">
         <v>87</v>
       </c>
       <c r="H23" s="49" t="s">
-        <v>661</v>
+        <v>653</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="32">
       <c r="A24" s="49" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="B24" s="49" t="s">
         <v>354</v>
       </c>
       <c r="C24" s="49" t="s">
-        <v>658</v>
+        <v>650</v>
       </c>
       <c r="D24" s="49" t="s">
-        <v>659</v>
+        <v>651</v>
       </c>
       <c r="E24" s="49" t="s">
         <v>347</v>
       </c>
       <c r="F24" s="49" t="s">
-        <v>662</v>
+        <v>654</v>
       </c>
       <c r="G24" s="49">
         <v>83</v>
       </c>
       <c r="H24" s="49" t="s">
-        <v>663</v>
+        <v>655</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="32">
       <c r="A25" s="49" t="s">
-        <v>619</v>
+        <v>611</v>
       </c>
       <c r="B25" s="49" t="s">
-        <v>620</v>
+        <v>612</v>
       </c>
       <c r="C25" s="49" t="s">
-        <v>658</v>
+        <v>650</v>
       </c>
       <c r="D25" s="49" t="s">
-        <v>659</v>
+        <v>651</v>
       </c>
       <c r="E25" s="49" t="s">
         <v>347</v>
       </c>
       <c r="F25" s="49" t="s">
-        <v>664</v>
+        <v>656</v>
       </c>
       <c r="G25" s="49">
         <v>89</v>
       </c>
       <c r="H25" s="49" t="s">
-        <v>663</v>
+        <v>655</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="32">
       <c r="A26" s="49" t="s">
-        <v>665</v>
+        <v>657</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>666</v>
+        <v>658</v>
       </c>
       <c r="C26" s="49" t="s">
-        <v>667</v>
+        <v>659</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>668</v>
+        <v>660</v>
       </c>
       <c r="E26" s="49" t="s">
         <v>347</v>
       </c>
       <c r="F26" s="49" t="s">
-        <v>669</v>
+        <v>661</v>
       </c>
       <c r="G26" s="49">
         <v>75</v>
       </c>
       <c r="H26" s="49" t="s">
-        <v>670</v>
+        <v>662</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="32">
       <c r="A27" s="49" t="s">
-        <v>671</v>
+        <v>663</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>672</v>
+        <v>664</v>
       </c>
       <c r="C27" s="49" t="s">
-        <v>673</v>
+        <v>665</v>
       </c>
       <c r="D27" s="49" t="s">
-        <v>668</v>
+        <v>660</v>
       </c>
       <c r="E27" s="49" t="s">
         <v>347</v>
       </c>
       <c r="F27" s="49" t="s">
-        <v>674</v>
+        <v>666</v>
       </c>
       <c r="G27" s="49">
         <v>27</v>
       </c>
       <c r="H27" s="49" t="s">
-        <v>661</v>
+        <v>653</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="16">
       <c r="A28" s="49" t="s">
-        <v>675</v>
+        <v>667</v>
       </c>
       <c r="B28" s="49" t="s">
-        <v>676</v>
+        <v>668</v>
       </c>
       <c r="C28" s="49" t="s">
-        <v>673</v>
+        <v>665</v>
       </c>
       <c r="D28" s="49" t="s">
-        <v>677</v>
+        <v>669</v>
       </c>
       <c r="E28" s="49" t="s">
         <v>334</v>
       </c>
       <c r="F28" s="49" t="s">
-        <v>659</v>
+        <v>651</v>
       </c>
       <c r="G28" s="49">
         <v>88</v>
       </c>
       <c r="H28" s="49" t="s">
-        <v>661</v>
+        <v>653</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="36">
       <c r="A30" s="50" t="s">
-        <v>678</v>
+        <v>670</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="16">
@@ -4570,81 +4682,81 @@
         <v>318</v>
       </c>
       <c r="C31" s="51" t="s">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="D31" s="51" t="s">
-        <v>680</v>
+        <v>672</v>
       </c>
       <c r="E31" s="51" t="s">
-        <v>681</v>
+        <v>673</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="16">
       <c r="A32" s="49" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="B32" s="49" t="s">
         <v>349</v>
       </c>
       <c r="C32" s="49" t="s">
-        <v>682</v>
+        <v>674</v>
       </c>
       <c r="D32" s="49" t="s">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="E32" s="49" t="s">
-        <v>684</v>
+        <v>676</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="16">
       <c r="A33" s="49" t="s">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="B33" s="49" t="s">
         <v>341</v>
       </c>
       <c r="C33" s="49" t="s">
-        <v>686</v>
+        <v>678</v>
       </c>
       <c r="D33" s="49" t="s">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="E33" s="49" t="s">
-        <v>688</v>
+        <v>680</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="16">
       <c r="A34" s="49" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="B34" s="49" t="s">
         <v>361</v>
       </c>
       <c r="C34" s="49" t="s">
-        <v>686</v>
+        <v>678</v>
       </c>
       <c r="D34" s="49" t="s">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="E34" s="49" t="s">
-        <v>690</v>
+        <v>682</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16">
       <c r="A35" s="49" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="B35" s="49" t="s">
         <v>354</v>
       </c>
       <c r="C35" s="49" t="s">
-        <v>686</v>
+        <v>678</v>
       </c>
       <c r="D35" s="49" t="s">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="E35" s="49" t="s">
-        <v>684</v>
+        <v>676</v>
       </c>
     </row>
   </sheetData>
@@ -4670,33 +4782,33 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>691</v>
+        <v>683</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>692</v>
+        <v>684</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>693</v>
+        <v>685</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>695</v>
+        <v>687</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>696</v>
+        <v>688</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>698</v>
+        <v>690</v>
       </c>
       <c r="C2" s="4">
         <v>250</v>
@@ -4705,19 +4817,19 @@
         <v>30</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>700</v>
+        <v>692</v>
       </c>
       <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="C3" s="4">
         <v>350</v>
@@ -4726,10 +4838,10 @@
         <v>100</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>700</v>
+        <v>692</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>347</v>
@@ -4737,10 +4849,10 @@
     </row>
     <row r="4" spans="1:7" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>704</v>
+        <v>696</v>
       </c>
       <c r="C4" s="4">
         <v>500</v>
@@ -4749,51 +4861,51 @@
         <v>250</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>700</v>
+        <v>692</v>
       </c>
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="C5" s="4">
         <v>750</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="G5" s="4"/>
     </row>
     <row r="8" spans="1:7" ht="17" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>321</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>712</v>
+        <v>704</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>278</v>
@@ -4801,138 +4913,138 @@
     </row>
     <row r="11" spans="1:7" ht="30" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>713</v>
+        <v>705</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>714</v>
+        <v>706</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>715</v>
+        <v>707</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>717</v>
+        <v>709</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="30" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="30" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="30" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>724</v>
+        <v>716</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>725</v>
+        <v>717</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>726</v>
+        <v>718</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>726</v>
+        <v>718</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>726</v>
+        <v>718</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
     </row>
   </sheetData>
@@ -4957,30 +5069,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>735</v>
+        <v>727</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="D2" s="4">
         <v>0</v>
@@ -4991,30 +5103,30 @@
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>739</v>
+        <v>731</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>740</v>
+        <v>732</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>741</v>
+        <v>733</v>
       </c>
       <c r="D3" s="4">
         <v>500</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>742</v>
+        <v>734</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>743</v>
+        <v>735</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>744</v>
+        <v>736</v>
       </c>
       <c r="D4" s="4">
         <v>0</v>
@@ -5050,36 +5162,36 @@
   <sheetData>
     <row r="1" spans="1:9" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>633</v>
+        <v>625</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>745</v>
+        <v>737</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>746</v>
+        <v>738</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>747</v>
+        <v>739</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>749</v>
+        <v>741</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>750</v>
+        <v>742</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>751</v>
+        <v>743</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>752</v>
+        <v>744</v>
       </c>
       <c r="B2" s="4">
         <v>3200</v>
@@ -5094,13 +5206,13 @@
         <v>225</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>753</v>
+        <v>745</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>754</v>
+        <v>746</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>755</v>
+        <v>747</v>
       </c>
       <c r="I2" s="4">
         <v>300</v>
@@ -5108,7 +5220,7 @@
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>756</v>
+        <v>748</v>
       </c>
       <c r="B3" s="4">
         <v>3800</v>
@@ -5123,13 +5235,13 @@
         <v>125</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>757</v>
+        <v>749</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>758</v>
+        <v>750</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>759</v>
+        <v>751</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>191</v>
@@ -5137,7 +5249,7 @@
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>760</v>
+        <v>752</v>
       </c>
       <c r="B4" s="4">
         <v>1200</v>
@@ -5152,13 +5264,13 @@
         <v>167</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>761</v>
+        <v>753</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>762</v>
+        <v>754</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>755</v>
+        <v>747</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>191</v>
@@ -5194,16 +5306,16 @@
         <v>320</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>763</v>
+        <v>755</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>764</v>
+        <v>756</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>765</v>
+        <v>757</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>766</v>
+        <v>758</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
@@ -5214,16 +5326,16 @@
         <v>350</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>767</v>
+        <v>759</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>191</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>768</v>
+        <v>760</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
@@ -5234,7 +5346,7 @@
         <v>337</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="D3" s="4">
         <v>2</v>
@@ -5243,7 +5355,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>769</v>
+        <v>761</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
@@ -5254,7 +5366,7 @@
         <v>343</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>770</v>
+        <v>762</v>
       </c>
       <c r="D4" s="4">
         <v>1</v>
@@ -5263,7 +5375,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>771</v>
+        <v>763</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
@@ -5274,7 +5386,7 @@
         <v>350</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="D5" s="4">
         <v>1</v>
@@ -5283,7 +5395,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>772</v>
+        <v>764</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
@@ -5294,7 +5406,7 @@
         <v>350</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="D6" s="4">
         <v>0</v>
@@ -5303,7 +5415,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>773</v>
+        <v>765</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
@@ -5314,7 +5426,7 @@
         <v>330</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
       <c r="D7" s="4">
         <v>0</v>
@@ -5323,7 +5435,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>774</v>
+        <v>766</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
@@ -5334,7 +5446,7 @@
         <v>350</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="D8" s="4">
         <v>0</v>
@@ -5343,7 +5455,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>775</v>
+        <v>767</v>
       </c>
     </row>
   </sheetData>
@@ -5593,66 +5705,66 @@
   <sheetData>
     <row r="1" spans="1:2" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>776</v>
+        <v>768</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>777</v>
+        <v>769</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>778</v>
+        <v>770</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>779</v>
+        <v>771</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>780</v>
+        <v>772</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>781</v>
+        <v>773</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>782</v>
+        <v>774</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>783</v>
+        <v>775</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>784</v>
+        <v>776</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>785</v>
+        <v>777</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>786</v>
+        <v>778</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>787</v>
+        <v>779</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>788</v>
+        <v>780</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>789</v>
+        <v>781</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>790</v>
+        <v>782</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>791</v>
+        <v>783</v>
       </c>
     </row>
   </sheetData>
@@ -5677,10 +5789,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>792</v>
+        <v>784</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>793</v>
+        <v>785</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>327</v>
@@ -5688,57 +5800,57 @@
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>794</v>
+        <v>786</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>795</v>
+        <v>787</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>796</v>
+        <v>788</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>797</v>
+        <v>789</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>798</v>
+        <v>790</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>797</v>
+        <v>789</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>800</v>
+        <v>792</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>801</v>
+        <v>793</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>797</v>
+        <v>789</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>803</v>
+        <v>795</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>804</v>
+        <v>796</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>805</v>
+        <v>797</v>
       </c>
     </row>
   </sheetData>
@@ -7572,114 +7684,216 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="48" customWidth="1"/>
-    <col min="3" max="3" width="80" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="77.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28" customHeight="1">
+    <row r="1" spans="1:3" ht="24" customHeight="1">
       <c r="A1" s="48" t="s">
         <v>371</v>
       </c>
       <c r="B1" s="48" t="s">
         <v>372</v>
       </c>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="54" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16">
-      <c r="A2" s="49" t="s">
+    <row r="2" spans="1:3" ht="24" customHeight="1">
+      <c r="A2" s="55" t="s">
         <v>374</v>
       </c>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="52" t="s">
+        <v>798</v>
+      </c>
+      <c r="C2" s="58" t="s">
         <v>375</v>
       </c>
-      <c r="C2" s="49" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1">
+      <c r="A3" s="56"/>
+      <c r="B3" s="52" t="s">
+        <v>799</v>
+      </c>
+      <c r="C3" s="59"/>
+    </row>
+    <row r="4" spans="1:3" ht="24" customHeight="1">
+      <c r="A4" s="57"/>
+      <c r="B4" s="52" t="s">
+        <v>354</v>
+      </c>
+      <c r="C4" s="60"/>
+    </row>
+    <row r="5" spans="1:3" ht="24" customHeight="1">
+      <c r="A5" s="55" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16">
-      <c r="A3" s="49" t="s">
+      <c r="B5" s="52" t="s">
+        <v>581</v>
+      </c>
+      <c r="C5" s="58" t="s">
         <v>377</v>
       </c>
-      <c r="B3" s="49" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="24" customHeight="1">
+      <c r="A6" s="56"/>
+      <c r="B6" s="52" t="s">
+        <v>587</v>
+      </c>
+      <c r="C6" s="59"/>
+    </row>
+    <row r="7" spans="1:3" ht="24" customHeight="1">
+      <c r="A7" s="57"/>
+      <c r="B7" s="52" t="s">
+        <v>582</v>
+      </c>
+      <c r="C7" s="60"/>
+    </row>
+    <row r="8" spans="1:3" ht="24" customHeight="1">
+      <c r="A8" s="55" t="s">
         <v>378</v>
       </c>
-      <c r="C3" s="49" t="s">
+      <c r="B8" s="52" t="s">
+        <v>519</v>
+      </c>
+      <c r="C8" s="58" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16">
-      <c r="A4" s="49" t="s">
+    <row r="9" spans="1:3" ht="24" customHeight="1">
+      <c r="A9" s="57"/>
+      <c r="B9" s="52" t="s">
+        <v>521</v>
+      </c>
+      <c r="C9" s="60"/>
+    </row>
+    <row r="10" spans="1:3" ht="24" customHeight="1">
+      <c r="A10" s="55" t="s">
         <v>380</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B10" s="52" t="s">
+        <v>448</v>
+      </c>
+      <c r="C10" s="58" t="s">
         <v>381</v>
       </c>
-      <c r="C4" s="49" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="24" customHeight="1">
+      <c r="A11" s="56"/>
+      <c r="B11" s="52" t="s">
+        <v>800</v>
+      </c>
+      <c r="C11" s="59"/>
+    </row>
+    <row r="12" spans="1:3" ht="24" customHeight="1">
+      <c r="A12" s="57"/>
+      <c r="B12" s="52" t="s">
+        <v>801</v>
+      </c>
+      <c r="C12" s="60"/>
+    </row>
+    <row r="13" spans="1:3" ht="24" customHeight="1">
+      <c r="A13" s="55" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="16">
-      <c r="A5" s="49" t="s">
+      <c r="B13" s="52" t="s">
+        <v>802</v>
+      </c>
+      <c r="C13" s="58" t="s">
         <v>383</v>
       </c>
-      <c r="B5" s="49" t="s">
+    </row>
+    <row r="14" spans="1:3" ht="24" customHeight="1">
+      <c r="A14" s="57"/>
+      <c r="B14" s="52">
+        <v>97433001001</v>
+      </c>
+      <c r="C14" s="60"/>
+    </row>
+    <row r="15" spans="1:3" ht="24" customHeight="1">
+      <c r="A15" s="55" t="s">
         <v>384</v>
       </c>
-      <c r="C5" s="49" t="s">
+      <c r="B15" s="52" t="s">
+        <v>803</v>
+      </c>
+      <c r="C15" s="58" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16">
-      <c r="A6" s="49" t="s">
+    <row r="16" spans="1:3" ht="24" customHeight="1">
+      <c r="A16" s="57"/>
+      <c r="B16" s="52" t="s">
+        <v>804</v>
+      </c>
+      <c r="C16" s="60"/>
+    </row>
+    <row r="17" spans="1:3" ht="24" customHeight="1">
+      <c r="A17" s="55" t="s">
         <v>386</v>
       </c>
-      <c r="B6" s="49" t="s">
+      <c r="B17" s="52" t="s">
+        <v>805</v>
+      </c>
+      <c r="C17" s="58" t="s">
         <v>387</v>
       </c>
-      <c r="C6" s="49" t="s">
+    </row>
+    <row r="18" spans="1:3" ht="24" customHeight="1">
+      <c r="A18" s="56"/>
+      <c r="B18" s="52" t="s">
+        <v>806</v>
+      </c>
+      <c r="C18" s="59"/>
+    </row>
+    <row r="19" spans="1:3" ht="24" customHeight="1">
+      <c r="A19" s="57"/>
+      <c r="B19" s="52" t="s">
+        <v>807</v>
+      </c>
+      <c r="C19" s="60"/>
+    </row>
+    <row r="20" spans="1:3" ht="24" customHeight="1">
+      <c r="A20" s="55" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16">
-      <c r="A7" s="49" t="s">
+      <c r="B20" s="52" t="s">
+        <v>808</v>
+      </c>
+      <c r="C20" s="58" t="s">
         <v>389</v>
       </c>
-      <c r="B7" s="49" t="s">
-        <v>390</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="16">
-      <c r="A8" s="49" t="s">
-        <v>392</v>
-      </c>
-      <c r="B8" s="49" t="s">
-        <v>393</v>
-      </c>
-      <c r="C8" s="49" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="16">
-      <c r="A9" s="49" t="s">
-        <v>395</v>
-      </c>
-      <c r="B9" s="49" t="s">
-        <v>396</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>397</v>
-      </c>
+    </row>
+    <row r="21" spans="1:3" ht="24" customHeight="1">
+      <c r="A21" s="57"/>
+      <c r="B21" s="53" t="s">
+        <v>809</v>
+      </c>
+      <c r="C21" s="60"/>
     </row>
   </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7697,22 +7911,22 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28" customHeight="1">
       <c r="A1" s="23" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="D1" s="24" t="s">
         <v>318</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="G1" s="23" t="s">
         <v>327</v>
@@ -7720,10 +7934,10 @@
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1">
       <c r="A2" s="25" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="C2" s="25" t="s">
         <v>362</v>
@@ -7732,13 +7946,13 @@
         <v>361</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="45" customHeight="1">
@@ -7755,13 +7969,13 @@
         <v>328</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>408</v>
+        <v>400</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="45" customHeight="1">
@@ -7769,7 +7983,7 @@
         <v>337</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="C4" s="25" t="s">
         <v>338</v>
@@ -7778,13 +7992,13 @@
         <v>336</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="45" customHeight="1">
@@ -7792,7 +8006,7 @@
         <v>343</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="C5" s="25" t="s">
         <v>344</v>
@@ -7801,13 +8015,13 @@
         <v>341</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="G5" s="25" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="45" customHeight="1">
@@ -7815,7 +8029,7 @@
         <v>343</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>368</v>
@@ -7824,21 +8038,21 @@
         <v>366</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="G6" s="25" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="45" customHeight="1">
       <c r="A7" s="25" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>351</v>
@@ -7847,21 +8061,21 @@
         <v>349</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" customHeight="1">
       <c r="A8" s="25" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>358</v>
@@ -7870,18 +8084,18 @@
         <v>357</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" customHeight="1">
       <c r="A9" s="25" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="B9" s="25" t="s">
         <v>367</v>
@@ -7893,13 +8107,13 @@
         <v>366</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -7929,56 +8143,56 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>318</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>349</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>436</v>
+        <v>428</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>440</v>
+        <v>432</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>341</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>191</v>
@@ -7989,56 +8203,56 @@
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>354</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>437</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>444</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>361</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>361</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>191</v>
@@ -8071,19 +8285,19 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>318</v>
@@ -8091,19 +8305,19 @@
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>333</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>349</v>
@@ -8111,19 +8325,19 @@
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>341</v>
@@ -8131,19 +8345,19 @@
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>361</v>
@@ -8151,19 +8365,19 @@
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>333</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>354</v>
@@ -8171,19 +8385,19 @@
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>333</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>357</v>
@@ -8191,25 +8405,25 @@
     </row>
     <row r="9" spans="1:6" ht="17" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="7" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="28" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>112</v>
@@ -8217,7 +8431,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>112</v>
@@ -8225,7 +8439,7 @@
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>112</v>
@@ -8233,7 +8447,7 @@
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>165</v>
@@ -8241,7 +8455,7 @@
     </row>
     <row r="17" spans="1:2" ht="30" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>112</v>
@@ -8249,39 +8463,39 @@
     </row>
     <row r="20" spans="1:2" ht="17" customHeight="1">
       <c r="A20" s="6" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="28" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>